<commit_message>
Update SQL Schema and add NoSQL Schema template.
</commit_message>
<xml_diff>
--- a/templates/db-schema/db-schema-sql.xlsx
+++ b/templates/db-schema/db-schema-sql.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hardik/Documents/Thynqit Repos/GitHub/bootcamp-foundational/templates/db-schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35BC885-9AE8-0644-8497-C66FC9DE68F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0D24BA2-0BF5-2F47-AEE2-D9DB7A98487D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19540" xr2:uid="{E33CE129-43D8-974C-BD8A-5178B14EA020}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
@@ -639,7 +639,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -666,6 +666,14 @@
       <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -852,10 +860,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -880,31 +889,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -912,30 +897,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -947,6 +908,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
@@ -961,11 +925,60 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1393,232 +1406,232 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="e" vm="1">
+      <c r="A1" s="32" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
+      <c r="A2" s="32"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
+      <c r="A3" s="32"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="32"/>
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="32"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="11"/>
+      <c r="A4" s="32"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="32"/>
+      <c r="M4" s="32"/>
+      <c r="N4" s="32"/>
+      <c r="O4" s="32"/>
+      <c r="P4" s="32"/>
+      <c r="Q4" s="32"/>
+      <c r="R4" s="32"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
+      <c r="A5" s="32"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="32"/>
+      <c r="N5" s="32"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="32"/>
+      <c r="Q5" s="32"/>
+      <c r="R5" s="32"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="11"/>
+      <c r="A6" s="32"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="32"/>
+      <c r="R6" s="32"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A7" s="21"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="26"/>
+      <c r="R7" s="26"/>
     </row>
     <row r="8" spans="1:18" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="33" t="s">
         <v>164</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="33"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="33"/>
+      <c r="N8" s="33"/>
+      <c r="O8" s="33"/>
+      <c r="P8" s="33"/>
+      <c r="Q8" s="33"/>
+      <c r="R8" s="33"/>
     </row>
     <row r="9" spans="1:18" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="10"/>
+      <c r="A9" s="33"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="33"/>
+      <c r="M9" s="33"/>
+      <c r="N9" s="33"/>
+      <c r="O9" s="33"/>
+      <c r="P9" s="33"/>
+      <c r="Q9" s="33"/>
+      <c r="R9" s="33"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="22"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22"/>
-      <c r="N10" s="22"/>
-      <c r="O10" s="22"/>
-      <c r="P10" s="22"/>
-      <c r="Q10" s="22"/>
-      <c r="R10" s="22"/>
+      <c r="A10" s="27"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="27"/>
+      <c r="N10" s="27"/>
+      <c r="O10" s="27"/>
+      <c r="P10" s="27"/>
+      <c r="Q10" s="27"/>
+      <c r="R10" s="27"/>
     </row>
     <row r="11" spans="1:18" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="15" t="s">
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="15"/>
-      <c r="O11" s="15"/>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="15"/>
-      <c r="R11" s="15"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="23"/>
+      <c r="P11" s="23"/>
+      <c r="Q11" s="23"/>
+      <c r="R11" s="23"/>
     </row>
     <row r="12" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
@@ -1627,777 +1640,886 @@
       <c r="B12" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="19"/>
       <c r="J12" s="1" t="s">
         <v>178</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="L12" s="24" t="s">
         <v>180</v>
       </c>
-      <c r="M12" s="14"/>
-      <c r="N12" s="12" t="s">
+      <c r="M12" s="25"/>
+      <c r="N12" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="O12" s="14"/>
+      <c r="O12" s="25"/>
       <c r="P12" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="Q12" s="12" t="s">
+      <c r="Q12" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="R12" s="14"/>
+      <c r="R12" s="25"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A13" s="16"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="24"/>
-      <c r="M13" s="25"/>
-      <c r="N13" s="24"/>
-      <c r="O13" s="25"/>
-      <c r="P13" s="17"/>
-      <c r="Q13" s="24"/>
-      <c r="R13" s="25"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="21"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="21"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="21"/>
+      <c r="R13" s="22"/>
     </row>
     <row r="14" spans="1:18" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="16">
-        <v>1</v>
-      </c>
-      <c r="B14" s="16" t="s">
+      <c r="A14" s="8">
+        <v>1</v>
+      </c>
+      <c r="B14" s="35" t="s">
         <v>168</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="33">
-        <v>1</v>
-      </c>
-      <c r="K14" s="33" t="s">
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="18">
+        <v>1</v>
+      </c>
+      <c r="K14" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="L14" s="28" t="s">
+      <c r="L14" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="M14" s="29"/>
-      <c r="N14" s="28" t="s">
+      <c r="M14" s="13"/>
+      <c r="N14" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="O14" s="29"/>
-      <c r="P14" s="33" t="s">
+      <c r="O14" s="13"/>
+      <c r="P14" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="Q14" s="28" t="s">
+      <c r="Q14" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="R14" s="29"/>
+      <c r="R14" s="13"/>
     </row>
     <row r="15" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="16">
+      <c r="A15" s="8">
         <v>2</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="28" t="s">
         <v>175</v>
       </c>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="30"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="30"/>
-      <c r="P15" s="23"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="30"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="19"/>
+      <c r="L15" s="14"/>
+      <c r="M15" s="15"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="15"/>
+      <c r="P15" s="19"/>
+      <c r="Q15" s="14"/>
+      <c r="R15" s="15"/>
     </row>
     <row r="16" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="16">
+      <c r="A16" s="8">
         <v>3</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="30"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="30"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="30"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="15"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="15"/>
     </row>
     <row r="17" spans="1:18" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="16">
+      <c r="A17" s="8">
         <v>4</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="28" t="s">
         <v>176</v>
       </c>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="31"/>
-      <c r="M17" s="32"/>
-      <c r="N17" s="31"/>
-      <c r="O17" s="32"/>
-      <c r="P17" s="34"/>
-      <c r="Q17" s="31"/>
-      <c r="R17" s="32"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="20"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="17"/>
     </row>
     <row r="18" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="16">
+      <c r="A18" s="8">
         <v>5</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="24"/>
-      <c r="M18" s="25"/>
-      <c r="N18" s="24"/>
-      <c r="O18" s="25"/>
-      <c r="P18" s="16"/>
-      <c r="Q18" s="24"/>
-      <c r="R18" s="25"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="21"/>
+      <c r="R18" s="22"/>
     </row>
     <row r="19" spans="1:18" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="16">
+      <c r="A19" s="8">
         <v>6</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="25"/>
-      <c r="N19" s="24"/>
-      <c r="O19" s="25"/>
-      <c r="P19" s="16"/>
-      <c r="Q19" s="24"/>
-      <c r="R19" s="25"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="22"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A20" s="16">
+      <c r="A20" s="8">
         <v>7</v>
       </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="16"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="25"/>
-      <c r="N20" s="24"/>
-      <c r="O20" s="25"/>
-      <c r="P20" s="16"/>
-      <c r="Q20" s="24"/>
-      <c r="R20" s="25"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="22"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="21"/>
+      <c r="R20" s="22"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="16">
+      <c r="A21" s="8">
         <v>8</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="23"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="16"/>
-      <c r="L21" s="24"/>
-      <c r="M21" s="25"/>
-      <c r="N21" s="24"/>
-      <c r="O21" s="25"/>
-      <c r="P21" s="16"/>
-      <c r="Q21" s="24"/>
-      <c r="R21" s="25"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="21"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="21"/>
+      <c r="O21" s="22"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="21"/>
+      <c r="R21" s="22"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="16">
+      <c r="A22" s="8">
         <v>9</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="23"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="16"/>
-      <c r="L22" s="24"/>
-      <c r="M22" s="25"/>
-      <c r="N22" s="24"/>
-      <c r="O22" s="25"/>
-      <c r="P22" s="16"/>
-      <c r="Q22" s="24"/>
-      <c r="R22" s="25"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="21"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="22"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="21"/>
+      <c r="R22" s="22"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A23" s="16">
+      <c r="A23" s="8">
         <v>10</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="16"/>
-      <c r="L23" s="24"/>
-      <c r="M23" s="25"/>
-      <c r="N23" s="24"/>
-      <c r="O23" s="25"/>
-      <c r="P23" s="16"/>
-      <c r="Q23" s="24"/>
-      <c r="R23" s="25"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="21"/>
+      <c r="M23" s="22"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="22"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="21"/>
+      <c r="R23" s="22"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A24" s="16">
+      <c r="A24" s="8">
         <v>11</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="23"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="16"/>
-      <c r="L24" s="24"/>
-      <c r="M24" s="25"/>
-      <c r="N24" s="24"/>
-      <c r="O24" s="25"/>
-      <c r="P24" s="16"/>
-      <c r="Q24" s="24"/>
-      <c r="R24" s="25"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="21"/>
+      <c r="M24" s="22"/>
+      <c r="N24" s="21"/>
+      <c r="O24" s="22"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="21"/>
+      <c r="R24" s="22"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A25" s="16">
+      <c r="A25" s="8">
         <v>12</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
-      <c r="L25" s="24"/>
-      <c r="M25" s="25"/>
-      <c r="N25" s="24"/>
-      <c r="O25" s="25"/>
-      <c r="P25" s="16"/>
-      <c r="Q25" s="24"/>
-      <c r="R25" s="25"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="21"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="21"/>
+      <c r="O25" s="22"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="21"/>
+      <c r="R25" s="22"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A26" s="16">
+      <c r="A26" s="8">
         <v>13</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="16"/>
-      <c r="K26" s="16"/>
-      <c r="L26" s="24"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="24"/>
-      <c r="O26" s="25"/>
-      <c r="P26" s="16"/>
-      <c r="Q26" s="24"/>
-      <c r="R26" s="25"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="21"/>
+      <c r="M26" s="22"/>
+      <c r="N26" s="21"/>
+      <c r="O26" s="22"/>
+      <c r="P26" s="8"/>
+      <c r="Q26" s="21"/>
+      <c r="R26" s="22"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A27" s="16">
+      <c r="A27" s="8">
         <v>14</v>
       </c>
-      <c r="B27" s="17"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
-      <c r="L27" s="24"/>
-      <c r="M27" s="25"/>
-      <c r="N27" s="24"/>
-      <c r="O27" s="25"/>
-      <c r="P27" s="16"/>
-      <c r="Q27" s="24"/>
-      <c r="R27" s="25"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="21"/>
+      <c r="M27" s="22"/>
+      <c r="N27" s="21"/>
+      <c r="O27" s="22"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="21"/>
+      <c r="R27" s="22"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A28" s="16">
+      <c r="A28" s="8">
         <v>15</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
-      <c r="L28" s="24"/>
-      <c r="M28" s="25"/>
-      <c r="N28" s="24"/>
-      <c r="O28" s="25"/>
-      <c r="P28" s="16"/>
-      <c r="Q28" s="24"/>
-      <c r="R28" s="25"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="21"/>
+      <c r="M28" s="22"/>
+      <c r="N28" s="21"/>
+      <c r="O28" s="22"/>
+      <c r="P28" s="8"/>
+      <c r="Q28" s="21"/>
+      <c r="R28" s="22"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A29" s="16">
+      <c r="A29" s="8">
         <v>16</v>
       </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="20"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="24"/>
-      <c r="M29" s="25"/>
-      <c r="N29" s="24"/>
-      <c r="O29" s="25"/>
-      <c r="P29" s="16"/>
-      <c r="Q29" s="24"/>
-      <c r="R29" s="25"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="21"/>
+      <c r="M29" s="22"/>
+      <c r="N29" s="21"/>
+      <c r="O29" s="22"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="21"/>
+      <c r="R29" s="22"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A30" s="16">
+      <c r="A30" s="8">
         <v>17</v>
       </c>
-      <c r="B30" s="17"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
-      <c r="L30" s="24"/>
-      <c r="M30" s="25"/>
-      <c r="N30" s="24"/>
-      <c r="O30" s="25"/>
-      <c r="P30" s="16"/>
-      <c r="Q30" s="24"/>
-      <c r="R30" s="25"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="21"/>
+      <c r="M30" s="22"/>
+      <c r="N30" s="21"/>
+      <c r="O30" s="22"/>
+      <c r="P30" s="8"/>
+      <c r="Q30" s="21"/>
+      <c r="R30" s="22"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A31" s="16">
+      <c r="A31" s="8">
         <v>18</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="16"/>
-      <c r="K31" s="16"/>
-      <c r="L31" s="24"/>
-      <c r="M31" s="25"/>
-      <c r="N31" s="24"/>
-      <c r="O31" s="25"/>
-      <c r="P31" s="16"/>
-      <c r="Q31" s="24"/>
-      <c r="R31" s="25"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="21"/>
+      <c r="M31" s="22"/>
+      <c r="N31" s="21"/>
+      <c r="O31" s="22"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="21"/>
+      <c r="R31" s="22"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A32" s="16">
+      <c r="A32" s="8">
         <v>19</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="20"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="16"/>
-      <c r="K32" s="16"/>
-      <c r="L32" s="24"/>
-      <c r="M32" s="25"/>
-      <c r="N32" s="24"/>
-      <c r="O32" s="25"/>
-      <c r="P32" s="16"/>
-      <c r="Q32" s="24"/>
-      <c r="R32" s="25"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="21"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="21"/>
+      <c r="O32" s="22"/>
+      <c r="P32" s="8"/>
+      <c r="Q32" s="21"/>
+      <c r="R32" s="22"/>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A33" s="16">
+      <c r="A33" s="8">
         <v>20</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="16"/>
-      <c r="K33" s="16"/>
-      <c r="L33" s="24"/>
-      <c r="M33" s="25"/>
-      <c r="N33" s="24"/>
-      <c r="O33" s="25"/>
-      <c r="P33" s="16"/>
-      <c r="Q33" s="24"/>
-      <c r="R33" s="25"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="21"/>
+      <c r="M33" s="22"/>
+      <c r="N33" s="21"/>
+      <c r="O33" s="22"/>
+      <c r="P33" s="8"/>
+      <c r="Q33" s="21"/>
+      <c r="R33" s="22"/>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A34" s="16">
+      <c r="A34" s="8">
         <v>21</v>
       </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="23"/>
-      <c r="J34" s="16"/>
-      <c r="K34" s="16"/>
-      <c r="L34" s="24"/>
-      <c r="M34" s="25"/>
-      <c r="N34" s="24"/>
-      <c r="O34" s="25"/>
-      <c r="P34" s="16"/>
-      <c r="Q34" s="24"/>
-      <c r="R34" s="25"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="30"/>
+      <c r="I34" s="19"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="21"/>
+      <c r="M34" s="22"/>
+      <c r="N34" s="21"/>
+      <c r="O34" s="22"/>
+      <c r="P34" s="8"/>
+      <c r="Q34" s="21"/>
+      <c r="R34" s="22"/>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A35" s="16">
-        <v>22</v>
-      </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="23"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="L35" s="24"/>
-      <c r="M35" s="25"/>
-      <c r="N35" s="24"/>
-      <c r="O35" s="25"/>
-      <c r="P35" s="16"/>
-      <c r="Q35" s="24"/>
-      <c r="R35" s="25"/>
+      <c r="A35" s="8">
+        <v>22</v>
+      </c>
+      <c r="B35" s="9"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="30"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="21"/>
+      <c r="M35" s="22"/>
+      <c r="N35" s="21"/>
+      <c r="O35" s="22"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="21"/>
+      <c r="R35" s="22"/>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A36" s="16">
+      <c r="A36" s="8">
         <v>23</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="16"/>
-      <c r="K36" s="16"/>
-      <c r="L36" s="24"/>
-      <c r="M36" s="25"/>
-      <c r="N36" s="24"/>
-      <c r="O36" s="25"/>
-      <c r="P36" s="16"/>
-      <c r="Q36" s="24"/>
-      <c r="R36" s="25"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="30"/>
+      <c r="I36" s="19"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="21"/>
+      <c r="M36" s="22"/>
+      <c r="N36" s="21"/>
+      <c r="O36" s="22"/>
+      <c r="P36" s="8"/>
+      <c r="Q36" s="21"/>
+      <c r="R36" s="22"/>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A37" s="16">
+      <c r="A37" s="8">
         <v>24</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="20"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="16"/>
-      <c r="K37" s="16"/>
-      <c r="L37" s="24"/>
-      <c r="M37" s="25"/>
-      <c r="N37" s="24"/>
-      <c r="O37" s="25"/>
-      <c r="P37" s="16"/>
-      <c r="Q37" s="24"/>
-      <c r="R37" s="25"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="29"/>
+      <c r="E37" s="29"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="30"/>
+      <c r="I37" s="19"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="21"/>
+      <c r="M37" s="22"/>
+      <c r="N37" s="21"/>
+      <c r="O37" s="22"/>
+      <c r="P37" s="8"/>
+      <c r="Q37" s="21"/>
+      <c r="R37" s="22"/>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A38" s="16">
+      <c r="A38" s="8">
         <v>25</v>
       </c>
-      <c r="B38" s="17"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="20"/>
-      <c r="I38" s="23"/>
-      <c r="J38" s="16"/>
-      <c r="K38" s="16"/>
-      <c r="L38" s="24"/>
-      <c r="M38" s="25"/>
-      <c r="N38" s="24"/>
-      <c r="O38" s="25"/>
-      <c r="P38" s="16"/>
-      <c r="Q38" s="24"/>
-      <c r="R38" s="25"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="30"/>
+      <c r="I38" s="19"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="21"/>
+      <c r="M38" s="22"/>
+      <c r="N38" s="21"/>
+      <c r="O38" s="22"/>
+      <c r="P38" s="8"/>
+      <c r="Q38" s="21"/>
+      <c r="R38" s="22"/>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A39" s="16">
+      <c r="A39" s="8">
         <v>26</v>
       </c>
-      <c r="B39" s="17"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="23"/>
-      <c r="J39" s="16"/>
-      <c r="K39" s="16"/>
-      <c r="L39" s="24"/>
-      <c r="M39" s="25"/>
-      <c r="N39" s="24"/>
-      <c r="O39" s="25"/>
-      <c r="P39" s="16"/>
-      <c r="Q39" s="24"/>
-      <c r="R39" s="25"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="29"/>
+      <c r="F39" s="29"/>
+      <c r="G39" s="29"/>
+      <c r="H39" s="30"/>
+      <c r="I39" s="19"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="21"/>
+      <c r="M39" s="22"/>
+      <c r="N39" s="21"/>
+      <c r="O39" s="22"/>
+      <c r="P39" s="8"/>
+      <c r="Q39" s="21"/>
+      <c r="R39" s="22"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A40" s="16">
+      <c r="A40" s="8">
         <v>27</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="16"/>
-      <c r="K40" s="16"/>
-      <c r="L40" s="24"/>
-      <c r="M40" s="25"/>
-      <c r="N40" s="24"/>
-      <c r="O40" s="25"/>
-      <c r="P40" s="16"/>
-      <c r="Q40" s="24"/>
-      <c r="R40" s="25"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="30"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="8"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="21"/>
+      <c r="M40" s="22"/>
+      <c r="N40" s="21"/>
+      <c r="O40" s="22"/>
+      <c r="P40" s="8"/>
+      <c r="Q40" s="21"/>
+      <c r="R40" s="22"/>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A41" s="16">
+      <c r="A41" s="8">
         <v>28</v>
       </c>
-      <c r="B41" s="17"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="20"/>
-      <c r="I41" s="23"/>
-      <c r="J41" s="16"/>
-      <c r="K41" s="16"/>
-      <c r="L41" s="26"/>
-      <c r="M41" s="27"/>
-      <c r="N41" s="26"/>
-      <c r="O41" s="27"/>
-      <c r="P41" s="16"/>
-      <c r="Q41" s="26"/>
-      <c r="R41" s="27"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="30"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="8"/>
+      <c r="K41" s="8"/>
+      <c r="L41" s="10"/>
+      <c r="M41" s="11"/>
+      <c r="N41" s="10"/>
+      <c r="O41" s="11"/>
+      <c r="P41" s="8"/>
+      <c r="Q41" s="10"/>
+      <c r="R41" s="11"/>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A42" s="16">
+      <c r="A42" s="8">
         <v>29</v>
       </c>
-      <c r="B42" s="17"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="19"/>
-      <c r="F42" s="19"/>
-      <c r="G42" s="19"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="23"/>
-      <c r="J42" s="16"/>
-      <c r="K42" s="16"/>
-      <c r="L42" s="26"/>
-      <c r="M42" s="27"/>
-      <c r="N42" s="26"/>
-      <c r="O42" s="27"/>
-      <c r="P42" s="16"/>
-      <c r="Q42" s="26"/>
-      <c r="R42" s="27"/>
+      <c r="B42" s="9"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="30"/>
+      <c r="I42" s="19"/>
+      <c r="J42" s="8"/>
+      <c r="K42" s="8"/>
+      <c r="L42" s="10"/>
+      <c r="M42" s="11"/>
+      <c r="N42" s="10"/>
+      <c r="O42" s="11"/>
+      <c r="P42" s="8"/>
+      <c r="Q42" s="10"/>
+      <c r="R42" s="11"/>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A43" s="16">
+      <c r="A43" s="8">
         <v>30</v>
       </c>
-      <c r="B43" s="17"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="19"/>
-      <c r="E43" s="19"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="19"/>
-      <c r="H43" s="20"/>
-      <c r="I43" s="23"/>
-      <c r="J43" s="16"/>
-      <c r="K43" s="16"/>
-      <c r="L43" s="26"/>
-      <c r="M43" s="27"/>
-      <c r="N43" s="26"/>
-      <c r="O43" s="27"/>
-      <c r="P43" s="16"/>
-      <c r="Q43" s="26"/>
-      <c r="R43" s="27"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="19"/>
+      <c r="J43" s="8"/>
+      <c r="K43" s="8"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="11"/>
+      <c r="N43" s="10"/>
+      <c r="O43" s="11"/>
+      <c r="P43" s="8"/>
+      <c r="Q43" s="10"/>
+      <c r="R43" s="11"/>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A44" s="16">
+      <c r="A44" s="8">
         <v>31</v>
       </c>
-      <c r="B44" s="17"/>
-      <c r="C44" s="18"/>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="19"/>
-      <c r="G44" s="19"/>
-      <c r="H44" s="20"/>
-      <c r="I44" s="23"/>
-      <c r="J44" s="16"/>
-      <c r="K44" s="16"/>
-      <c r="L44" s="26"/>
-      <c r="M44" s="27"/>
-      <c r="N44" s="26"/>
-      <c r="O44" s="27"/>
-      <c r="P44" s="16"/>
-      <c r="Q44" s="26"/>
-      <c r="R44" s="27"/>
+      <c r="B44" s="9"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="29"/>
+      <c r="H44" s="30"/>
+      <c r="I44" s="19"/>
+      <c r="J44" s="8"/>
+      <c r="K44" s="8"/>
+      <c r="L44" s="10"/>
+      <c r="M44" s="11"/>
+      <c r="N44" s="10"/>
+      <c r="O44" s="11"/>
+      <c r="P44" s="8"/>
+      <c r="Q44" s="10"/>
+      <c r="R44" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="133">
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="C13:H13"/>
+    <mergeCell ref="C14:H14"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:R6"/>
+    <mergeCell ref="A8:R9"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="C15:H15"/>
+    <mergeCell ref="C16:H16"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="J11:R11"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="A7:R7"/>
+    <mergeCell ref="A10:R10"/>
+    <mergeCell ref="I11:I44"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="C42:H42"/>
+    <mergeCell ref="C43:H43"/>
+    <mergeCell ref="C44:H44"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="L36:M36"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="N41:O41"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="N43:O43"/>
+    <mergeCell ref="N44:O44"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q23:R23"/>
     <mergeCell ref="Q42:R42"/>
     <mergeCell ref="Q43:R43"/>
     <mergeCell ref="Q44:R44"/>
@@ -2422,116 +2544,15 @@
     <mergeCell ref="Q24:R24"/>
     <mergeCell ref="Q25:R25"/>
     <mergeCell ref="Q26:R26"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="Q29:R29"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="N43:O43"/>
-    <mergeCell ref="N44:O44"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="L39:M39"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="L33:M33"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="L35:M35"/>
-    <mergeCell ref="L36:M36"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="L38:M38"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="L29:M29"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="J11:R11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="A7:R7"/>
-    <mergeCell ref="A10:R10"/>
-    <mergeCell ref="I11:I44"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="C42:H42"/>
-    <mergeCell ref="C43:H43"/>
-    <mergeCell ref="C44:H44"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="C28:H28"/>
-    <mergeCell ref="C29:H29"/>
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="C31:H31"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="C15:H15"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="C17:H17"/>
-    <mergeCell ref="C18:H18"/>
-    <mergeCell ref="C19:H19"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="C13:H13"/>
-    <mergeCell ref="C14:H14"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A1:R6"/>
-    <mergeCell ref="A8:R9"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B14" location="users!A1" display="users" xr:uid="{5755E9B5-5325-F648-B591-4C9FD23E1484}"/>
+    <hyperlink ref="B15" location="trips!A1" display="trips" xr:uid="{7F64F2B5-0325-0846-AF6D-E765A4994836}"/>
+    <hyperlink ref="B16" location="vehicles!A1" display="vehicles" xr:uid="{37A027EE-72CC-C44B-B01D-C1027B521809}"/>
+    <hyperlink ref="B17" location="payments!A1" display="payments" xr:uid="{8F822A9B-F116-5245-BAE5-F152A7689C19}"/>
+    <hyperlink ref="B18" location="offers!A1" display="offers" xr:uid="{629398A4-2041-924C-A506-2FB6A64C931D}"/>
+    <hyperlink ref="B19" location="addresses!A1" display="addresses" xr:uid="{AFE74BC0-517C-F24E-8251-BE2DE6123803}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2555,33 +2576,33 @@
       <c r="A1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -3027,33 +3048,33 @@
       <c r="A1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -3464,7 +3485,7 @@
       <c r="H17" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="7">
         <v>0</v>
       </c>
       <c r="J17" s="3" t="s">
@@ -3531,33 +3552,33 @@
       <c r="A1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -4035,33 +4056,33 @@
       <c r="A1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -4178,7 +4199,7 @@
       <c r="H8" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="7">
         <v>0</v>
       </c>
       <c r="J8" s="3" t="s">
@@ -4338,7 +4359,7 @@
       <c r="H13" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="7">
         <v>0</v>
       </c>
       <c r="J13" s="3" t="s">
@@ -4370,7 +4391,7 @@
       <c r="H14" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="7">
         <v>0</v>
       </c>
       <c r="J14" s="3" t="s">
@@ -4469,33 +4490,33 @@
       <c r="A1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -4787,33 +4808,33 @@
       <c r="A1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="34" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="34" t="s">
         <v>136</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">

</xml_diff>